<commit_message>
Refresh PatchPad QC report
</commit_message>
<xml_diff>
--- a/PatchPad_Editor_QC.xlsx
+++ b/PatchPad_Editor_QC.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="138" customWidth="1" min="1" max="1"/>
@@ -558,7 +558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fresh first-level QC after local fixes.</t>
+          <t>Fresh first-level QC after rubric compression and undo fixes.</t>
         </is>
       </c>
     </row>
@@ -649,131 +649,138 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Local QC fixes resolved the static packaging and prompt/rubric issues; the remaining blocker is run validation.</t>
+          <t>Static QC is clean after fixes; the remaining blocker is run validation.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Fixed in this pass</t>
+          <t>Fixed before this pass</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Removed generated task-tree artifacts: node_modules, committed SQLite DB/WAL/SHM files, local server logs, .patchpad-server.job, and tests/__pycache__.</t>
+          <t>Compressed browser rubric from 32 criteria to 20 criteria.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Clarified instruction.md so saving unchanged content must not create a duplicate revision.</t>
+          <t>Reweighted simple merged criteria to 0.5, hard undo/multi-caret criteria to 2.0, and revision restore to 1.5.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Clarified instruction.md so find controls cycle through matches, matching the Find Next wrap verifier.</t>
+          <t>Fixed contiguous typing undo grouping so one Undo reverses a typed word.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Made solution/app/run-local.cmd resolve paths relative to itself instead of hardcoding C:\Users\abc.</t>
+          <t>Fixed selection replacement typing and multi-caret typed insertion to use the same grouped undo behavior.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Adjusted the browser verifier prompt to re-establish intended document/editor state where practical before each criterion, reducing cascade risk.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+          <t>Confirmed revision restore is implemented as an unsaved dirty draft with a single pre-restore undo snapshot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Removed brittle apt/Node package pins from the Dockerfile to avoid Daytona sandbox build failures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Found clean after fixes</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Required Harbor files are present: instruction.md, task.toml, environment/Dockerfile, solution/solve.sh, tests/test.sh.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>task.toml and browser.toml parse successfully with Python tomllib.</t>
+          <t>Required Harbor files are present: instruction.md, task.toml, environment/Dockerfile, solution/solve.sh, tests/test.sh.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>Rubric has 32 criteria, all weighted between 0.5 and 2.0, with no zero-weight criteria; total raw weight is 43.5.</t>
+          <t>task.toml and browser.toml parse successfully with Python tomllib.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>tests/test.py writes an initial 0.0 reward floor and catches BaseException; tests/test.sh also writes fallback reward files if Python exits before writing them.</t>
+          <t>Rubric has 20 criteria, all weighted between 0.5 and 2.0, with no zero-weight criteria; total raw weight is 15.5.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Verifier prompt explicitly tells the judge not to trust APP_MANIFEST.md as grading evidence.</t>
+          <t>tests/test.py writes an initial 0.0 reward floor and catches BaseException; tests/test.sh also writes fallback reward files if Python exits before writing them.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Server-side conflict and tampering checks exist via direct in-page fetch probes, not only UI button checks.</t>
+          <t>Verifier prompt explicitly tells the judge not to trust APP_MANIFEST.md as grading evidence.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Golden JavaScript files pass syntax checks with Node: src/index.js, src/db.js, and public/js/app.js.</t>
+          <t>Server-side conflict and tampering checks exist via direct in-page fetch probes, not only UI button checks.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>Dockerfile pins the Ubuntu base digest and most key tool/package versions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+          <t>Node-based JavaScript syntax re-check could not be repeated in this shell because node is not currently available on PATH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Upload zip has executable solve.sh/test.sh and contains no node_modules, DB files, logs, caches, or pyc files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Checks not run</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>Full Oracle RewardKit browser run was not executed in this first-level pass.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Full Oracle RewardKit browser run was not executed in this first-level pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>No model run spread was available, so the target of Oracle 1.0 and model score below 0.7 is unproven.</t>
         </is>
@@ -897,7 +904,7 @@
       </c>
       <c r="F2" s="11" t="inlineStr">
         <is>
-          <t>The skill treats Oracle score 1.0 as the proof that the task is solvable. Static checks cannot establish that RewardKit, Playwright MCP, and the golden pass all 32 criteria end to end.</t>
+          <t>The QC skill treats Oracle score 1.0 as the proof that the task is solvable. Static checks cannot establish that RewardKit, Playwright MCP, and the golden pass all 20 criteria end to end.</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Document browser verifier protocol guidance
</commit_message>
<xml_diff>
--- a/PatchPad_Editor_QC.xlsx
+++ b/PatchPad_Editor_QC.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PatchPad Editor" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Run Evidence" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PatchPad" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PatchPad Editor'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PatchPad'!$A$1:$L$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="8">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,7 +61,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="009C6500"/>
+      <color rgb="009C0006"/>
       <sz val="10"/>
     </font>
     <font>
@@ -67,8 +70,26 @@
       <color rgb="009C0006"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +121,11 @@
         <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -127,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -155,18 +181,33 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -534,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="138" customWidth="1" min="1" max="1"/>
@@ -551,21 +592,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PatchPad Editor - Harbor Task QC</t>
+          <t>PatchPad Editor — Harbor Task QC</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fresh first-level QC after rubric compression and undo fixes.</t>
+          <t>Fresh QC of patchpad-editor.zip with GPT-5.6-SOL run job-b7a904c5 (trial task__AGHJ6TP). No Oracle job was provided.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Scope: static package/prompt/rubric/golden checks only. No Oracle/model RewardKit run artifacts were present under patchpad-editor.</t>
+          <t>QC per harbor-task-qc skill. Focus on defects that distort the training signal. Packaging/layout and reward-on-crash paths were checked.</t>
         </is>
       </c>
     </row>
@@ -619,170 +660,119 @@
     <row r="6" ht="62" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>PatchPad Editor</t>
+          <t>PatchPad</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>1</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>Static QC is clean after fixes; the remaining blocker is run validation.</t>
+      <c r="H6" s="11" t="n">
+        <v>0.7097</v>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>Changes requested: heaviest undo criteria grade unstated contiguous-typing coalescing. GPT 0.71 is partly measuring a missing brief line, not just capability.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Fixed before this pass</t>
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Overall verdict</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>Compressed browser rubric from 32 criteria to 20 criteria.</t>
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>CHANGES REQUESTED — The GPT 0.7097 score is dominated by three undo criteria (4.5/15.5 weight ≈ 29%) that enforce editor undo grouping the brief never states.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>Reweighted simple merged criteria to 0.5, hard undo/multi-caret criteria to 2.0, and revision restore to 1.5.</t>
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>instruction.md explicitly requires atomic undo for paste, cut, and multi-caret edits — but never says contiguous typing (or type-to-replace) is one undo step. The golden implements typingGroup coalescing; the rubric grades that private convention.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Fixed contiguous typing undo grouping so one Undo reverses a typed word.</t>
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>No Oracle trial was in the delivered job zip, so solvability is not run-proven (golden exists and looks coherent).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Fixed selection replacement typing and multi-caret typed insertion to use the same grouped undo behavior.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Confirmed revision restore is implemented as an unsaved dirty draft with a single pre-restore undo snapshot.</t>
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Otherwise the task looks solid: proper zip root, custom-editor prohibition stated, conflict/save probes graded, GPT passed 17/20 including multi-caret, stale-save, and server persistence.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Removed brittle apt/Node package pins from the Dockerfile to avoid Daytona sandbox build failures.</t>
+          <t>What was checked and found clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Zip packages as patchpad-editor/ with 0 __MACOSX; solve.sh and test.sh mode 755.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Found clean after fixes</t>
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Required Harbor layout; unified instruction.md; OPENROUTER only in [verifier.env]; no prompts/ leak.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>Required Harbor files are present: instruction.md, task.toml, environment/Dockerfile, solution/solve.sh, tests/test.sh.</t>
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>test.py writes placeholder reward then BaseException handler; test.sh writes reward if python never did.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>task.toml and browser.toml parse successfully with Python tomllib.</t>
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Seed markers (Northwind title, TODO, ALPHA-*, OMEGA-END-ANCHOR) live in /assets/incident_seed.json copied into the agent image — agent-visible, not rubric-only leakage.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>Rubric has 20 criteria, all weighted between 0.5 and 2.0, with no zero-weight criteria; total raw weight is 15.5.</t>
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Reward math: criteria weights sum 15.5; GPT earned 11.0 → 11/15.5 = 0.709677 ≈ 0.7097.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>tests/test.py writes an initial 0.0 reward floor and catches BaseException; tests/test.sh also writes fallback reward files if Python exits before writing them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>Verifier prompt explicitly tells the judge not to trust APP_MANIFEST.md as grading evidence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>Server-side conflict and tampering checks exist via direct in-page fetch probes, not only UI button checks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>Node-based JavaScript syntax re-check could not be repeated in this shell because node is not currently available on PATH.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>Upload zip has executable solve.sh/test.sh and contains no node_modules, DB files, logs, caches, or pyc files.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Checks not run</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
-        <is>
-          <t>Full Oracle RewardKit browser run was not executed in this first-level pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>No model run spread was available, so the target of Oracle 1.0 and model score below 0.7 is unproven.</t>
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>GPT failures are app undo behavior (per-keystroke), not harness timeouts or action-errors. graded=1, no_op=0.</t>
         </is>
       </c>
     </row>
@@ -797,7 +787,108 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="84" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Run evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>From each trial's result.json, verifier/agentic.json, report.json and screenshots/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Model / agent</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Reward</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Prog</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Agent s</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Verifier s</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>patchpad-editor</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>GPT-5.6-SOL</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>0.7097</v>
+      </c>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n">
+        <v>545</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>3326</v>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>job-b7a904c5 / twenty-verifiers / task__AGHJ6TP — 17/20 criteria, graded=1, no_op=0. All 3 fails are undo-granularity criteria (weights 2.0+0.5+2.0).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -877,67 +968,241 @@
       </c>
     </row>
     <row r="2" ht="100" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>PP-01</t>
-        </is>
-      </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>PP-001</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>instruction.md Editor behavior (undo bullets); tests/rubric/browser/browser.toml undo_contiguous_typing_group (weight 2.0)</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Rubric requires: type contiguous word TYPING-GROUP-CHECK, one Undo removes the whole word, one Redo restores it. instruction.md never states that contiguous typing is one undoable edit.</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>Classic graded-but-not-stated. The brief DOES require atomic undo for paste, cut, and multi-caret — which makes the omission of typing-group coalescing look deliberate and invites per-keystroke undo as a reasonable reading. difficulty_explanation mentions undo granularity, but that text is not the agent brief.</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>Correct implementations that undo character-by-character lose weight 2.0 (~13% of total). GPT failed exactly this way: 'each Undo removes exactly one character'. Corrupts the training signal toward the golden's private typingGroup convention.</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>Add one bullet to instruction.md, e.g. 'Contiguous typing without moving the caret is one undoable edit (one Undo removes the whole typed run).' Keep the rubric as-is once stated.</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>GPT reward-details undo_contiguous_typing_group: value 0.0 — per-keystroke undo reproduced repeatedly. Instruction lines on undo only mention paste, cut, and multi-caret as atomic. Golden app.js uses state.typingGroup / pushGroupedUndo for single-char inserts.</t>
+        </is>
+      </c>
+      <c r="J2" s="18" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr"/>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="100" customHeight="1">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>PP-002</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
-        <is>
-          <t>Run Validation</t>
-        </is>
-      </c>
-      <c r="D2" s="11" t="inlineStr">
-        <is>
-          <t>patchpad-editor/</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>No Harbor run artifacts were found under the task folder. run_inventory.py reported: "No trials found under patchpad-editor."</t>
-        </is>
-      </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>The QC skill treats Oracle score 1.0 as the proof that the task is solvable. Static checks cannot establish that RewardKit, Playwright MCP, and the golden pass all 20 criteria end to end.</t>
-        </is>
-      </c>
-      <c r="G2" s="11" t="inlineStr">
-        <is>
-          <t>The task should not be considered delivery-ready until Oracle scores 1.0 and representative model runs show the intended score spread.</t>
-        </is>
-      </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
-          <t>Run Oracle and at least the planned model set, then re-run QC in run-validation mode with result.json, reward.json, report.json, and agentic.json artifacts.</t>
-        </is>
-      </c>
-      <c r="I2" s="11" t="inlineStr">
-        <is>
-          <t>CONFIRMED: bundled run_inventory.py found no trials at depths 1-3.</t>
-        </is>
-      </c>
-      <c r="J2" s="16" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>instruction.md; browser.toml undo_paste_cut_replace_atomic (weight 2.0)</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Criterion requires paste, cut, AND type-to-replace each to be one undo step. Instruction states paste and cut as one undoable edit, but only says users can 'replace selected text by typing' — not that one Undo restores the original selection.</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>Judge confirmed paste and cut were atomic on the GPT app; the criterion still failed solely on the replace-by-typing sub-check, which shares the unstated typing-group rule from PP-001.</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>Another weight 2.0 (~13%) lost for an understated rule. Bundling a stated check (paste/cut) with an unstated one (replace atomic) makes the failure look like a full compound-edit miss.</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>State that replacing a selection by typing is one undoable edit, or split replace into its own criterion / drop it from this id until stated.</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>GPT reasoning: 'Paste and cut are each undone/redone atomically… However, the replace sub-check … is NOT atomic: one Undo only removes the last typed character.'</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="inlineStr">
         <is>
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="K2" s="11" t="inlineStr"/>
-      <c r="L2" s="11" t="inlineStr">
+      <c r="K3" s="12" t="inlineStr"/>
+      <c r="L3" s="12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="100" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>PP-003</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Verifier-Strictness</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>browser.toml undo_separate_locations_and_redo_clear (weight 0.5)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>This criterion failed on GPT because undo is per-keystroke, so LOCATION-ONE/TWO/THREE cannot each be one undo step. Redo-clear-on-new-edit was not independently disproven.</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Downstream of PP-001. Also, instruction never states that edits at separate caret locations are separate undo steps, nor that typing after Undo clears the Redo stack.</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>Extra 0.5 weight (~3%) lost as cascade/understatement rather than an independent measured defect.</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>After stating typing groups (PP-001), keep this criterion; also add one line that a new edit after Undo clears Redo.</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>GPT reasoning explicitly attributes the fail to the same per-keystroke root cause as undo_contiguous_typing_group.</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr"/>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="100" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>PP-004</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Delivered jobs: only job-b7a904c5 (OpenHands GPT-5.6-SOL). No oracle trial in zip.</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>QC package includes a model run (reward 0.7097) but no Oracle/solve.sh run scoring 1.0.</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Harbor QC requires an Oracle at 1.0 to prove the task is solvable. Absence means delivery readiness cannot be run-validated — only inferred from the golden.</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Client cannot confirm the golden passes its own verifier under the real harness. Any golden/rubric mismatch would ship undetected.</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Attach an Oracle job with reward 1.0 before client delivery, or re-run harbor oracle against this zip and include the trial.</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>job-b7a904c5 contains a single trial task__AGHJ6TP with agent openhands / openai/gpt-5.6-sol. Job stats n_total_trials=1. No oracle agent_info anywhere under the zip.</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
+        <is>
+          <t>NOT EXERCISED</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr"/>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:L5"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2 L3 L4 L5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Closed,Open,In progress,Won't fix,Verify at packaging"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>